<commit_message>
Log EDC image renames (EDC_* to TS105_*) in TikTok tracking sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Listings" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SKUs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Banned Words" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How To Use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Images" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Banned Words" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="How To Use" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1141,7 +1142,6 @@
       <c r="I3" t="n">
         <v>16</v>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1185,7 +1185,6 @@
       <c r="I4" t="n">
         <v>16</v>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1325,7 +1324,6 @@
       <c r="I7" t="n">
         <v>16</v>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1417,7 +1415,6 @@
       <c r="I9" t="n">
         <v>16</v>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1461,7 +1458,6 @@
       <c r="I10" t="n">
         <v>16</v>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1649,7 +1645,6 @@
       <c r="I14" t="n">
         <v>16</v>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1693,7 +1688,6 @@
       <c r="I15" t="n">
         <v>16</v>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1785,7 +1779,6 @@
       <c r="I17" t="n">
         <v>16</v>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1829,7 +1822,6 @@
       <c r="I18" t="n">
         <v>16</v>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1873,7 +1865,6 @@
       <c r="I19" t="n">
         <v>16</v>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1965,7 +1956,6 @@
       <c r="I21" t="n">
         <v>16</v>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2009,7 +1999,6 @@
       <c r="I22" t="n">
         <v>16</v>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2053,7 +2042,6 @@
       <c r="I23" t="n">
         <v>16</v>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2097,7 +2085,6 @@
       <c r="I24" t="n">
         <v>16</v>
       </c>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3485,6 +3472,322 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="n"/>
+      <c r="B1" s="3" t="n"/>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Shopify product</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Media ID</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OLD filename</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NEW filename</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>New URL</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Renamed on</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TS105</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EDC Rave Sprout (8835658776754)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>35270274973874</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EDC_1106.jpg</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TS105_01.jpg</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_01.jpg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TS105</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EDC Rave Sprout (8835658776754)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>35270323732658</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>EDC_1112.jpg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TS105_02.jpg</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_02.jpg</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TS105</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EDC Rave Sprout (8835658776754)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>35270275039410</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>EDC_1109.jpg</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TS105_03.jpg</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_03.jpg</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TS105</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EDC Rave Sprout (8835658776754)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>35270275006642</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>EDC_1107.jpg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>TS105_04.jpg</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_04.jpg</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TS105</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EDC Rave Sprout (8835658776754)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>35270275072178</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>EDC_1110.jpg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>TS105_05.jpg</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_05.jpg</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TS105</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EDC Rave Sprout (8835658776754)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>35270274941106</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>EDC_1114.jpg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TS105_06.jpg</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_06.jpg</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3886,7 +4189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix blank header row on Images tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -59,7 +59,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -70,6 +70,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3477,7 +3478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3491,54 +3492,84 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="n"/>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Shopify product</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Media ID</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>OLD filename</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>NEW filename</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>New URL</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Renamed on</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>TS105</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Shopify product</t>
+          <t>EDC Rave Sprout (8835658776754)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Media ID</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Position</t>
-        </is>
+          <t>35270274973874</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OLD filename</t>
+          <t>EDC_1106.jpg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NEW filename</t>
+          <t>TS105_01.jpg</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>New URL</t>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_01.jpg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Renamed on</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3555,25 +3586,25 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>35270274973874</t>
+          <t>35270323732658</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EDC_1106.jpg</t>
+          <t>EDC_1112.jpg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TS105_01.jpg</t>
+          <t>TS105_02.jpg</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_01.jpg</t>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_02.jpg</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -3595,25 +3626,25 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35270323732658</t>
+          <t>35270275039410</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>EDC_1112.jpg</t>
+          <t>EDC_1109.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TS105_02.jpg</t>
+          <t>TS105_03.jpg</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_02.jpg</t>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_03.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -3635,25 +3666,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>35270275039410</t>
+          <t>35270275006642</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>EDC_1109.jpg</t>
+          <t>EDC_1107.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TS105_03.jpg</t>
+          <t>TS105_04.jpg</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_03.jpg</t>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_04.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -3675,25 +3706,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>35270275006642</t>
+          <t>35270275072178</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EDC_1107.jpg</t>
+          <t>EDC_1110.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TS105_04.jpg</t>
+          <t>TS105_05.jpg</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_04.jpg</t>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_05.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3715,68 +3746,28 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>35270275072178</t>
+          <t>35270274941106</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EDC_1110.jpg</t>
+          <t>EDC_1114.jpg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TS105_05.jpg</t>
+          <t>TS105_06.jpg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_05.jpg</t>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_06.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TS105</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>EDC Rave Sprout (8835658776754)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>35270274941106</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>EDC_1114.jpg</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>TS105_06.jpg</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS105_06.jpg</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Log EDC alt text cleanup in TikTok tracking sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -59,7 +59,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -71,6 +71,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3478,7 +3481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3489,6 +3492,8 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3532,6 +3537,16 @@
           <t>Renamed on</t>
         </is>
       </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>OLD alt text</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>NEW alt text</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3572,6 +3587,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Three EDC rave sprout spring clips on white display steps — neon green hot pink, orange purple, and neon yellow turquoise colors</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Three neon rave sprout spring clips on white display steps — neon green hot pink, orange purple, and neon yellow turquoise colors</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3612,6 +3637,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Two EDC rave sprout spring clips in orange purple and neon yellow turquoise colors on a black flat-bill hat with white Las Vegas text</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Two neon rave sprout spring clips in orange purple and neon yellow turquoise colors on a black flat-bill hat</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3652,6 +3687,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>EDC rave sprout in neon green and hot pink — 3D printed festival hair clip and kandi charm</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Neon rave sprout in neon green and hot pink — 3D printed festival hair clip and kandi charm</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3692,6 +3737,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>EDC rave sprout spring clip hair accessory in orange and purple — fan-made kandi charm for EDC</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Neon rave sprout spring clip hair accessory in orange and purple — 3D printed kandi charm</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3732,6 +3787,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>EDC rave sprout fan-made festival hair clip in neon yellow and dark teal - limited edition EDC Las Vegas</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Neon rave sprout festival hair clip in neon yellow and dark teal</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3770,6 +3835,16 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>EDC rave sprout festival accessories clipped on festival hat showing multi colors — kandi bead charm and rave hair clip handmade</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Neon rave sprout festival accessories clipped on a festival hat showing multi colors — kandi bead charm and rave hair clip, handmade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new-listing CSV for TS101, TS103, TS105 relists; mark them delete-and-relist in tracking sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>1. Edit in place (in upload file)</t>
+          <t>4. Delete and relist</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
@@ -654,7 +654,7 @@
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Design is the artist's logo: TikTok image scanning may still flag it. Old TikTok SKUs repeated (NTMRE_1, _2, _3 each used twice); new SKUs are unique. Price spread $3 to $60.</t>
+          <t>Old listing DELETED 2026-10-21. Relist from TikTok_New_Listings_Pilot.csv. Design is the artist's logo: TikTok image scanning may still flag it. Old TikTok SKUs repeated (NTMRE_1, _2, _3 each used twice); new SKUs are unique. Price spread $3 to $60.</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>1. Edit in place (in upload file)</t>
+          <t>4. Delete and relist</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -814,7 +814,7 @@
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>10-pack only, $28 (list $30), matches Shopify WKN2 10-pack price. Description keeps TikTok's '10 pieces per pack' (no bonus promised). 'Trippy' is a placeholder descriptor.</t>
+          <t>Old listing DELETED 2026-10-21. Relist from TikTok_New_Listings_Pilot.csv. 10-pack only, $28 (list $30), matches Shopify WKN2 10-pack price. Description keeps TikTok's '10 pieces per pack' (no bonus promised). 'Trippy' is a placeholder descriptor.</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>2. Fix and resubmit (appeal)</t>
+          <t>4. Delete and relist</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
@@ -974,7 +974,7 @@
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>NOT IN TIKTOK'S BULK EXPORT (not live). Edit by hand in Seller Center. Frozen listings usually point to an IP/brand flag. Shopify copy says the design is a 'bold EDC logo', so renaming alone is unlikely to unfreeze it. Old SKUs start with EDC1 (the festival name itself).</t>
+          <t>Relist from TikTok_New_Listings_Pilot.csv (images renamed TS105_01-06 in Shopify). NOT IN TIKTOK'S BULK EXPORT (not live). Edit by hand in Seller Center. Frozen listings usually point to an IP/brand flag. Shopify copy says the design is a 'bold EDC logo', so renaming alone is unlikely to unfreeze it. Old SKUs start with EDC1 (the festival name itself).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use renamed Shopify photos (TS101_*, TS103_*) in TikTok create upload; log renames
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -3481,7 +3481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3845,6 +3845,606 @@
       <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Neon rave sprout festival accessories clipped on a festival hat showing multi colors — kandi bead charm and rave hair clip, handmade</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TS101</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NGTHMRE Logo Rave Sprout (8584861810866)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>35147504484530</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NGHTMRE_0060.jpg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TS101_01.jpg</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS101_01.jpg</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TS101</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NGTHMRE Logo Rave Sprout (8584861810866)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>35147504418994</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NGHTMRE_0061.jpg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TS101_02.jpg</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS101_02.jpg</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TS101</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NGTHMRE Logo Rave Sprout (8584861810866)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>35147504451762</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NGHTMRE_0063.jpg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TS101_03.jpg</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS101_03.jpg</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TS101</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NGTHMRE Logo Rave Sprout (8584861810866)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>35147504517298</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NGHTMRE_0059.jpg</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TS101_04.jpg</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS101_04.jpg</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TS101</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NGTHMRE Logo Rave Sprout (8584861810866)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>35147504550066</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>NGHTMRE_0058.jpg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TS101_05.jpg</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS101_05.jpg</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>35147120017586</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0616.jpg</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TS103_01.jpg</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_01.jpg</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>35147120083122</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0619.jpg</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TS103_02.jpg</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_02.jpg</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>35147120050354</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0618.jpg</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TS103_03.jpg</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_03.jpg</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>35147119952050</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0614.jpg</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TS103_04.jpg</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_04.jpg</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>35147119919282</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0613.jpg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>TS103_05.jpg</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_05.jpg</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>35147211505842</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0555.jpg</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TS103_06.jpg</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_06.jpg</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TS103</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Wakaan Drip Rave Sprout (8802402664626)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>35147211538610</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Liquid-Stranger-Drip_0557.jpg</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>TS103_07.jpg</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0726/0202/6162/files/TS103_07.jpg</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>(blank, unchanged)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename TikTok pack variants to 11/22/27/33 Pack and drop FREE/bonus wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -624,11 +624,11 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Clip a bold statement onto your hat, hair, or pashmina. This 3D printed rave sprout pairs a crisp graphic charm with a bouncy metal spring that moves with every beat.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Blue, Silk Purple, Black, or Rainbow&lt;/li&gt;&lt;li&gt;Packs: single, or 10- and 25-packs with bonus sprouts for gifting your whole crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Clip a bold statement onto your hat, hair, or pashmina. This 3D printed rave sprout pairs a crisp graphic charm with a bouncy metal spring that moves with every beat.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Blue, Silk Purple, Black, or Rainbow&lt;/li&gt;&lt;li&gt;Packs: single, 11-pack, or 27-pack, perfect for gifting your whole crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Trippy Rave Sprout 10 Pack | Festival Hat Clips &amp; Kandi Charms | Pink, Emerald, Orchid, Multicolor</t>
+          <t>Trippy Rave Sprout 11 Pack | Festival Hat Clips &amp; Kandi Charms | Pink, Emerald, Orchid, Multicolor</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
@@ -784,11 +784,11 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Stock up for the whole crew with a 10-pack of trippy rave sprouts in bold colors, ready for trading, gifting, or surprising a new friend at the show.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Emerald, Medium Orchid, or Multicolor&lt;/li&gt;&lt;li&gt;Quantity: 10 pieces per pack&lt;/li&gt;&lt;li&gt;Material: PLA plastic with a metal spring alligator clip&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Stock up for the whole crew with an 11-pack of trippy rave sprouts in bold colors, ready for trading, gifting, or surprising a new friend at the show.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Emerald, Medium Orchid, or Multicolor&lt;/li&gt;&lt;li&gt;Quantity: 11 pieces per pack&lt;/li&gt;&lt;li&gt;Material: PLA plastic with a metal spring alligator clip&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>578</v>
+        <v>588</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -944,11 +944,11 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Bright neon colors made for the main stage. This 3D printed rave sprout bounces on a metal spring clip with every beat and grips tight to hats, hair, and festival outfits. Vivid neon tones pop under blacklights and lasers all weekend. A built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece so you can keep the memory after the music stops. Weather-resistant adhesive holds up through desert heat and packed crowds. Choose Neon Green, Orange, Yellow, or Multicolor as a single or a 10-, 20-, or 30-pack with bonus sprouts for trading.</t>
+          <t>&lt;p&gt;Bright neon colors made for the main stage. This 3D printed rave sprout bounces on a metal spring clip with every beat, and its vivid neon tones pop under blacklights and lasers all weekend.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Neon Green, Orange, Yellow, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: single, 11-pack, 22-pack, or 33-pack for trading&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>555</v>
+        <v>595</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1055,6 +1055,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>TikTok variant name (relist)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1103,6 +1108,11 @@
           <t>Old SKU was used on two variants; 1 Pack: pricing-flag risk next to big packs</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1146,6 +1156,11 @@
       <c r="I3" t="n">
         <v>16</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1189,6 +1204,11 @@
       <c r="I4" t="n">
         <v>16</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>27 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1237,6 +1257,11 @@
           <t>Old SKU was used on two variants; 1 Pack: pricing-flag risk next to big packs</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1285,6 +1310,11 @@
           <t>Old SKU was used on two variants</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1328,6 +1358,11 @@
       <c r="I7" t="n">
         <v>16</v>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>27 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1376,6 +1411,11 @@
           <t>Old SKU was used on two variants; 1 Pack: pricing-flag risk next to big packs</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>1 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1419,6 +1459,11 @@
       <c r="I9" t="n">
         <v>16</v>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1462,6 +1507,11 @@
       <c r="I10" t="n">
         <v>16</v>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>27 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1510,6 +1560,11 @@
           <t>Old SKU was used on two variants</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1558,6 +1613,11 @@
           <t>Old SKU was used on two variants</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>27 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1960,6 +2020,11 @@
       <c r="I21" t="n">
         <v>16</v>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>11 Pack (color only)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2003,6 +2068,11 @@
       <c r="I22" t="n">
         <v>16</v>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>11 Pack (color only)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2046,6 +2116,11 @@
       <c r="I23" t="n">
         <v>16</v>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>11 Pack (color only)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2089,6 +2164,11 @@
       <c r="I24" t="n">
         <v>16</v>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>11 Pack (color only)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2797,6 +2877,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok; 1 Pack: pricing-flag risk next to big packs</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>1 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2845,6 +2930,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2893,6 +2983,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>22 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2941,6 +3036,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>33 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2989,6 +3089,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok; 1 Pack: pricing-flag risk next to big packs</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>1 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3037,6 +3142,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3085,6 +3195,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>22 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3133,6 +3248,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>33 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3181,6 +3301,11 @@
           <t>Old code YLTR is a flagged typo in Platform_Reference; new SKU uses YELW; TikTok listing has 8 SKUs: delete rows that aren't on TikTok; 1 Pack: pricing-flag risk next to big packs</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>1 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3229,6 +3354,11 @@
           <t>Old code YLTR is a flagged typo in Platform_Reference; new SKU uses YELW; TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3277,6 +3407,11 @@
           <t>Old code YLTR is a flagged typo in Platform_Reference; new SKU uses YELW; TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>22 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3325,6 +3460,11 @@
           <t>Old code YLTR is a flagged typo in Platform_Reference; new SKU uses YELW; TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>33 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3373,6 +3513,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>11 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3421,6 +3566,11 @@
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>22 Pack</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3467,6 +3617,11 @@
       <c r="J54" t="inlineStr">
         <is>
           <t>TikTok listing has 8 SKUs: delete rows that aren't on TikTok</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>33 Pack</t>
         </is>
       </c>
     </row>
@@ -4861,7 +5016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4964,6 +5119,18 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TikTok variant names drop "+ (N FREE)": 10+1 = 11 Pack, 20+2 = 22 Pack, 25+2 = 27 Pack, 30+3 = 33 Pack. Shopify names and all SKUs are unchanged. TikTok_New_Listings_Pilot.csv is outdated; use TikTok_Create_Pilot_3_Listings.xlsx.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log new TikTok product IDs for relisted TS101, TS103, TS105
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Live (8/8/2026)</t>
+          <t>RELISTED - Live 2026-10-21 (old: Live (8/8/2026))</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -648,8 +648,16 @@
           <t>https://shop.tiktok.com/view/product/1731695024946713558</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>1732777435658228694</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.tiktok.com/view/product/1732777435658228694 (verify)</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr">
@@ -751,7 +759,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Live (7/28/2026)</t>
+          <t>RELISTED - Live 2026-10-21 (old: Live (7/28/2026))</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -808,8 +816,16 @@
           <t>https://shop.tiktok.com/view/product/1732355495878497238</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>1732777435658097622</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.tiktok.com/view/product/1732777435658097622 (verify)</t>
+        </is>
+      </c>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr">
@@ -911,7 +927,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Frozen by platform (Tue)</t>
+          <t>RELISTED - Live 2026-10-21 (old: Frozen by platform (Tue))</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -968,8 +984,16 @@
           <t>https://shop.tiktok.com/view/product/1732394839248770006</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>1732777435658163158</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.tiktok.com/view/product/1732777435658163158 (verify)</t>
+        </is>
+      </c>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record CED variant links for TS101, TS103, TS105
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -662,7 +662,7 @@
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Old listing DELETED 2026-10-21. Relist from TikTok_New_Listings_Pilot.csv. Design is the artist's logo: TikTok image scanning may still flag it. Old TikTok SKUs repeated (NTMRE_1, _2, _3 each used twice); new SKUs are unique. Price spread $3 to $60.</t>
+          <t>All variants linked to Shopify in CED 2026-10-21 (manual link; title/description sync off, price/inventory sync on). Old listing DELETED 2026-10-21. Relist from TikTok_New_Listings_Pilot.csv. Design is the artist's logo: TikTok image scanning may still flag it. Old TikTok SKUs repeated (NTMRE_1, _2, _3 each used twice); new SKUs are unique. Price spread $3 to $60.</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Old listing DELETED 2026-10-21. Relist from TikTok_New_Listings_Pilot.csv. 10-pack only, $28 (list $30), matches Shopify WKN2 10-pack price. Description keeps TikTok's '10 pieces per pack' (no bonus promised). 'Trippy' is a placeholder descriptor.</t>
+          <t>All variants linked to Shopify in CED 2026-10-21 (manual link; title/description sync off, price/inventory sync on). Old listing DELETED 2026-10-21. Relist from TikTok_New_Listings_Pilot.csv. 10-pack only, $28 (list $30), matches Shopify WKN2 10-pack price. Description keeps TikTok's '10 pieces per pack' (no bonus promised). 'Trippy' is a placeholder descriptor.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Relist from TikTok_New_Listings_Pilot.csv (images renamed TS105_01-06 in Shopify). NOT IN TIKTOK'S BULK EXPORT (not live). Edit by hand in Seller Center. Frozen listings usually point to an IP/brand flag. Shopify copy says the design is a 'bold EDC logo', so renaming alone is unlikely to unfreeze it. Old SKUs start with EDC1 (the festival name itself).</t>
+          <t>All variants linked to Shopify in CED 2026-10-21 (manual link; title/description sync off, price/inventory sync on). Relist from TikTok_New_Listings_Pilot.csv (images renamed TS105_01-06 in Shopify). NOT IN TIKTOK'S BULK EXPORT (not live). Edit by hand in Seller Center. Frozen listings usually point to an IP/brand flag. Shopify copy says the design is a 'bold EDC logo', so renaming alone is unlikely to unfreeze it. Old SKUs start with EDC1 (the festival name itself).</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1084,6 +1084,11 @@
           <t>TikTok variant name (relist)</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Linked in CED (2026-10-21)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1137,6 +1142,11 @@
           <t>1 Pack</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_BLUE_PCK1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1185,6 +1195,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_BLUE_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1233,6 +1248,11 @@
           <t>27 Pack</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_BLUE_PCK25</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1286,6 +1306,11 @@
           <t>1 Pack</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_SLPL_PCK1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1339,6 +1364,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_SLPL_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1387,6 +1417,11 @@
           <t>27 Pack</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_SLPL_PCK25</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1440,6 +1475,11 @@
           <t>1 Pack</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_BLCK_PCK1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1488,6 +1528,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_BLCK_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1536,6 +1581,11 @@
           <t>27 Pack</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_BLCK_PCK25</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1589,6 +1639,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_MLTC_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1642,6 +1697,11 @@
           <t>27 Pack</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Yes -&gt; NGTH_MLTC_PCK25</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2049,6 +2109,11 @@
           <t>11 Pack (color only)</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Yes -&gt; WKN2_CPNK_PCK10 (color pairing guessed)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2097,6 +2162,11 @@
           <t>11 Pack (color only)</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Yes -&gt; WKN2_TRQS_PCK10 (color pairing guessed)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2145,6 +2215,11 @@
           <t>11 Pack (color only)</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Yes -&gt; WKN2_SLPL_PCK10 (color pairing guessed)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2193,6 +2268,11 @@
           <t>11 Pack (color only)</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Yes -&gt; WKN2_MLTC_PCK10 (color pairing guessed)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2906,6 +2986,11 @@
           <t>1 Pack</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_NGPK_PCK1</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2959,6 +3044,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_NGPK_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3012,6 +3102,11 @@
           <t>22 Pack</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_NGPK_PCK20</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3065,6 +3160,11 @@
           <t>33 Pack</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_NGPK_PCK30</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3118,6 +3218,11 @@
           <t>1 Pack</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_ORPL_PCK1</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3171,6 +3276,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_ORPL_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3224,6 +3334,11 @@
           <t>22 Pack</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_ORPL_PCK20</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3277,6 +3392,11 @@
           <t>33 Pack</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_ORPL_PCK30</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3330,6 +3450,11 @@
           <t>1 Pack</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_YLTR_PCK1</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3383,6 +3508,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_YLTR_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3436,6 +3566,11 @@
           <t>22 Pack</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_YLTR_PCK20</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3489,6 +3624,11 @@
           <t>33 Pack</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_YLTR_PCK30</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3542,6 +3682,11 @@
           <t>11 Pack</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_MLTC_PCK10</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3595,6 +3740,11 @@
           <t>22 Pack</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_MLTC_PCK20</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3646,6 +3796,11 @@
       <c r="K54" t="inlineStr">
         <is>
           <t>33 Pack</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Yes -&gt; EDC1_MLTC_PCK30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark Wakaan color pairings as confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -2111,7 +2111,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Yes -&gt; WKN2_CPNK_PCK10 (color pairing guessed)</t>
+          <t>Yes -&gt; WKN2_CPNK_PCK10 (color pairing confirmed by owner 2026-10-22)</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Yes -&gt; WKN2_TRQS_PCK10 (color pairing guessed)</t>
+          <t>Yes -&gt; WKN2_TRQS_PCK10 (color pairing confirmed by owner 2026-10-22)</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Yes -&gt; WKN2_SLPL_PCK10 (color pairing guessed)</t>
+          <t>Yes -&gt; WKN2_SLPL_PCK10 (color pairing confirmed by owner 2026-10-22)</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Yes -&gt; WKN2_MLTC_PCK10 (color pairing guessed)</t>
+          <t>Yes -&gt; WKN2_MLTC_PCK10 (color pairing confirmed by owner 2026-10-22)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 2: log 13 new TikTok product IDs after submit for review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -7088,14 +7088,11 @@
           <t>TS119_01.jpg</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7126,14 +7123,11 @@
           <t>TS119_02.jpg</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7164,14 +7158,11 @@
           <t>TS119_03.jpg</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7202,14 +7193,11 @@
           <t>TS119_04.jpg</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7240,14 +7228,11 @@
           <t>TS119_05.jpg</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7278,14 +7263,11 @@
           <t>TS120_01.jpg</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7316,14 +7298,11 @@
           <t>TS120_02.jpg</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7354,14 +7333,11 @@
           <t>TS120_03.jpg</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7392,14 +7368,11 @@
           <t>TS120_04.jpg</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7430,14 +7403,11 @@
           <t>TS121_01.jpg</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7468,14 +7438,11 @@
           <t>TS121_02.jpg</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7506,14 +7473,11 @@
           <t>TS121_03.jpg</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7544,14 +7508,11 @@
           <t>TS121_04.jpg</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7582,14 +7543,11 @@
           <t>TS121_05.jpg</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7620,14 +7578,11 @@
           <t>TS121_06.jpg</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7658,14 +7613,11 @@
           <t>TS121_07.jpg</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8279,7 +8231,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -8292,7 +8244,11 @@
           <t>&lt;p&gt;Spread the good vibes with funky 3D printed rave sprouts made for trading and gifting at every show.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Blue, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1732780426613527510</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Shopify's 15 variants at Shopify prices (TikTok had 8).</t>
@@ -8317,7 +8273,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -8330,7 +8286,11 @@
           <t>&lt;p&gt;Bring a little retro bass energy to your festival hat with this bold 3D printed rave sprout.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Green, Pink, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1732780426613986262</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Was filed under Stickers on TikTok.</t>
@@ -8368,8 +8328,6 @@
           <t>&lt;p&gt;Turn heads on the dance floor with this bold lettered rave sprout, 3D printed in punchy festival colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Silk Purple, Neon Green, Blue, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8402,8 +8360,6 @@
           <t>&lt;p&gt;Made for the emotional drops and singalong moments, this 3D printed rave sprout brings melodic bass vibes to any outfit.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Black, Orange, Neon Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8436,8 +8392,6 @@
           <t>&lt;p&gt;A bold bones emblem rave sprout for the funky, feel-good side of the festival, 3D printed and ready to trade.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Neon Green, Yellow, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8470,8 +8424,6 @@
           <t>&lt;p&gt;A cheeky party bunny rave sprout for the ravers who are always ready to send it, 3D printed in bright festival colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Blue, Pink, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8491,7 +8443,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -8504,8 +8456,11 @@
           <t>&lt;p&gt;Graffiti-style lettering meets bass music energy in this 3D printed rave sprout, mounted on a black spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Neon Green, Pink, Purple, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1732780426614051798</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8525,7 +8480,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -8538,8 +8493,11 @@
           <t>&lt;p&gt;A bold icon rave sprout for the house and techno crowd, 3D printed and mounted on a bouncy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Red, White, Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1732780426613593046</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8559,7 +8517,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -8572,7 +8530,11 @@
           <t>&lt;p&gt;Earthy greens and browns for the campground and the main stage alike, 3D printed and mounted on a metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Neon Green, White-Olive Green, Brown, Black, Olive Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1732780426613658582</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>Shopify's 17 variants (TikTok had 4 singles).</t>
@@ -8597,7 +8559,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8610,7 +8572,11 @@
           <t>&lt;p&gt;A dark, heavy text rave sprout for the headbangers in the front row, 3D printed and built for the pit.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1732780426613724118</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Shopify's 3 packs (TikTok had one 10 pack).</t>
@@ -8635,7 +8601,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8648,8 +8614,11 @@
           <t>&lt;p&gt;Built for bassheads who live for the wobble, this 3D printed rave sprout brings heavy festival energy to your hat or hair.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Orange, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1732780426613789654</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8669,7 +8638,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -8682,8 +8651,11 @@
           <t>&lt;p&gt;A cosmic, otherworldly rave sprout for the deep-bass crowd, 3D printed and mounted on a sturdy spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Silk Purple, Pink, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1732780426614117334</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8703,7 +8675,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -8716,7 +8688,11 @@
           <t>&lt;p&gt;A menacing masked face rave sprout for heavy bass nights, 3D printed in high detail and mounted on a metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1732780426613855190</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Shopify's 3 packs (TikTok had one single).</t>
@@ -8741,7 +8717,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -8754,7 +8730,11 @@
           <t>&lt;p&gt;A funky little creature rave sprout full of future-funk attitude, 3D printed in detail and ready for your festival hat.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 5 Pack, 11 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1732780426613920726</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Was filed under Figurines on TikTok.</t>
@@ -8779,7 +8759,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -8792,7 +8772,11 @@
           <t>&lt;p&gt;For the ravers who love strings, keys and soaring melodic drops, this dreamy 3D printed rave sprout brings the feels to any outfit.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: White, Yellow, Blue, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1732780426613461974</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Replacement added 2026-10-22. Was filed under Figurines on TikTok.</t>
@@ -8817,7 +8801,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -8830,7 +8814,11 @@
           <t>&lt;p&gt;An endless infinity loop design for the deep-bass crowd, 3D printed in bold colors and mounted on a sturdy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Cyan, Black, Orange, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1732780426614182870</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Replacement added 2026-10-22. Shopify stock shows 997-999 on some variants; check.</t>
@@ -8855,7 +8843,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>In TikTok_Create_Batch2_v2_13_Listings.xlsx (old listing deleted)</t>
+          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -8868,7 +8856,11 @@
           <t>&lt;p&gt;A cheeky hand gesture rave sprout with plenty of attitude, 3D printed and mounted on a bouncy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Red, White, Purple, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1732780426614248406</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Replacement added 2026-10-22. TikTok had 10-packs only; Shopify's 11 variants used.</t>
@@ -9006,7 +8998,6 @@
           <t>TS104_PINK_PCK1</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9055,7 +9046,6 @@
           <t>TS104_PINK_PCK10</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9104,7 +9094,6 @@
           <t>TS104_PINK_PCK20</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9153,7 +9142,6 @@
           <t>TS104_PINK_PCK30</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9202,7 +9190,6 @@
           <t>TS104_BLUE_PCK1</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9251,7 +9238,6 @@
           <t>TS104_BLUE_PCK10</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9300,7 +9286,6 @@
           <t>TS104_BLUE_PCK20</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9349,7 +9334,6 @@
           <t>TS104_BLUE_PCK30</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9398,7 +9382,6 @@
           <t>TS104_WHIT_PCK1</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9447,7 +9430,6 @@
           <t>TS104_WHIT_PCK10</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9496,7 +9478,6 @@
           <t>TS104_WHIT_PCK20</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9545,7 +9526,6 @@
           <t>TS104_WHIT_PCK30</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9594,7 +9574,6 @@
           <t>TS104_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9643,7 +9622,6 @@
           <t>TS104_MLTC_PCK20</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9692,7 +9670,6 @@
           <t>TS104_MLTC_PCK30</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9741,7 +9718,6 @@
           <t>TS106_YELW_PCK1</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9790,7 +9766,6 @@
           <t>TS106_YELW_PCK10</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9839,7 +9814,6 @@
           <t>TS106_YELW_PCK20</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9888,7 +9862,6 @@
           <t>TS106_YELW_PCK30</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9937,7 +9910,6 @@
           <t>TS106_GREN_PCK1</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9986,7 +9958,6 @@
           <t>TS106_GREN_PCK10</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -10035,7 +10006,6 @@
           <t>TS106_GREN_PCK20</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10084,7 +10054,6 @@
           <t>TS106_GREN_PCK30</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -10133,7 +10102,6 @@
           <t>TS106_PINK_PCK1</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10182,7 +10150,6 @@
           <t>TS106_PINK_PCK10</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10231,7 +10198,6 @@
           <t>TS106_PINK_PCK20</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10280,7 +10246,6 @@
           <t>TS106_PINK_PCK30</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10329,7 +10294,6 @@
           <t>TS106_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10378,7 +10342,6 @@
           <t>TS106_MLTC_PCK20</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10427,7 +10390,6 @@
           <t>TS106_MLTC_PCK30</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10476,7 +10438,6 @@
           <t>TS111_NGRN_PCK1</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10525,7 +10486,6 @@
           <t>TS111_NGRN_PCK10</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10574,7 +10534,6 @@
           <t>TS111_NGRN_PCK25</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10623,7 +10582,6 @@
           <t>TS111_NGRN_PCK40</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10672,7 +10630,6 @@
           <t>TS111_PINK_PCK1</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10721,7 +10678,6 @@
           <t>TS111_PINK_PCK10</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10770,7 +10726,6 @@
           <t>TS111_PINK_PCK25</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10819,7 +10774,6 @@
           <t>TS111_PINK_PCK40</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -10868,7 +10822,6 @@
           <t>TS111_PRPL_PCK1</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -10917,7 +10870,6 @@
           <t>TS111_PRPL_PCK10</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -10966,7 +10918,6 @@
           <t>TS111_PRPL_PCK25</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -11015,7 +10966,6 @@
           <t>TS111_PRPL_PCK40</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -11064,7 +11014,6 @@
           <t>TS111_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -11113,7 +11062,6 @@
           <t>TS111_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -11162,7 +11110,6 @@
           <t>TS111_MLTC_PCK40</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -11211,7 +11158,6 @@
           <t>TS112_REDD_PCK1</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11260,7 +11206,6 @@
           <t>TS112_REDD_PCK10</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11309,7 +11254,6 @@
           <t>TS112_REDD_PCK25</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11358,7 +11302,6 @@
           <t>TS112_WHIT_PCK1</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11407,7 +11350,6 @@
           <t>TS112_WHIT_PCK10</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11456,7 +11398,6 @@
           <t>TS112_WHIT_PCK25</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11505,7 +11446,6 @@
           <t>TS112_GREN_PCK1</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -11554,7 +11494,6 @@
           <t>TS112_GREN_PCK10</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11603,7 +11542,6 @@
           <t>TS112_GREN_PCK25</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11652,7 +11590,6 @@
           <t>TS112_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11701,7 +11638,6 @@
           <t>TS112_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11750,7 +11686,6 @@
           <t>TS113_NGRN_PCK1</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -11799,7 +11734,6 @@
           <t>TS113_NGRN_PCK10</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -11848,7 +11782,6 @@
           <t>TS113_NGRN_PCK25</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11897,7 +11830,6 @@
           <t>TS113_WOVG_PCK1</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -11946,7 +11878,6 @@
           <t>TS113_WOVG_PCK10</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11995,7 +11926,6 @@
           <t>TS113_WOVG_PCK25</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12044,7 +11974,6 @@
           <t>TS113_BRWN_PCK1</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12093,7 +12022,6 @@
           <t>TS113_BRWN_PCK10</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -12142,7 +12070,6 @@
           <t>TS113_BRWN_PCK25</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -12191,7 +12118,6 @@
           <t>TS113_BLCK_PCK1</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -12240,7 +12166,6 @@
           <t>TS113_BLCK_PCK10</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12289,7 +12214,6 @@
           <t>TS113_BLCK_PCK25</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12338,7 +12262,6 @@
           <t>TS113_OLVG_PCK1</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12387,7 +12310,6 @@
           <t>TS113_OLVG_PCK10</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12436,7 +12358,6 @@
           <t>TS113_OLVG_PCK25</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12485,7 +12406,6 @@
           <t>TS113_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12534,7 +12454,6 @@
           <t>TS113_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12552,7 +12471,6 @@
           <t>8584856010930</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>1 Pack</t>
@@ -12579,7 +12497,6 @@
           <t>TS114_PCK1</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -12597,7 +12514,6 @@
           <t>8584856010930</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>10 Pack + (1 FREE)</t>
@@ -12624,7 +12540,6 @@
           <t>TS114_PCK10</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -12642,7 +12557,6 @@
           <t>8584856010930</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>25 Pack + (2 FREE)</t>
@@ -12669,7 +12583,6 @@
           <t>TS114_PCK25</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -12718,7 +12631,6 @@
           <t>TS115_YELW_PCK1</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -12767,7 +12679,6 @@
           <t>TS115_YELW_PCK10</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -12816,7 +12727,6 @@
           <t>TS115_YELW_PCK25</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -12865,7 +12775,6 @@
           <t>TS115_YELW_PCK40</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -12914,7 +12823,6 @@
           <t>TS115_ORGN_PCK1</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -12963,7 +12871,6 @@
           <t>TS115_ORGN_PCK10</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -13012,7 +12919,6 @@
           <t>TS115_ORGN_PCK25</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -13061,7 +12967,6 @@
           <t>TS115_ORGN_PCK40</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13110,7 +13015,6 @@
           <t>TS115_WHIT_PCK1</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13159,7 +13063,6 @@
           <t>TS115_WHIT_PCK10</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -13208,7 +13111,6 @@
           <t>TS115_WHIT_PCK25</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13257,7 +13159,6 @@
           <t>TS115_WHIT_PCK40</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -13306,7 +13207,6 @@
           <t>TS115_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -13355,7 +13255,6 @@
           <t>TS115_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -13404,7 +13303,6 @@
           <t>TS115_MLTC_PCK40</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -13453,7 +13351,6 @@
           <t>TS116_SLPL_PCK1</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13502,7 +13399,6 @@
           <t>TS116_SLPL_PCK10</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -13551,7 +13447,6 @@
           <t>TS116_SLPL_PCK25</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -13600,7 +13495,6 @@
           <t>TS116_PINK_PCK1</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -13649,7 +13543,6 @@
           <t>TS116_PINK_PCK10</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13698,7 +13591,6 @@
           <t>TS116_PINK_PCK25</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -13747,7 +13639,6 @@
           <t>TS116_BLCK_PCK1</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -13796,7 +13687,6 @@
           <t>TS116_BLCK_PCK10</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13845,7 +13735,6 @@
           <t>TS116_BLCK_PCK25</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -13894,7 +13783,6 @@
           <t>TS116_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -13943,7 +13831,6 @@
           <t>TS116_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -13961,7 +13848,6 @@
           <t>8584856764594</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>1 Pack</t>
@@ -13988,7 +13874,6 @@
           <t>TS117_PCK1</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -14006,7 +13891,6 @@
           <t>8584856764594</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
           <t>10 Pack + (1 FREE)</t>
@@ -14033,7 +13917,6 @@
           <t>TS117_PCK10</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -14051,7 +13934,6 @@
           <t>8584856764594</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
           <t>25 Pack + (2 FREE)</t>
@@ -14078,7 +13960,6 @@
           <t>TS117_PCK25</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -14096,7 +13977,6 @@
           <t>8741157961906</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>1 Pack</t>
@@ -14123,7 +14003,6 @@
           <t>TS118_PCK1</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -14141,7 +14020,6 @@
           <t>8741157961906</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>5 Pack</t>
@@ -14168,7 +14046,6 @@
           <t>TS118_PCK5</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -14186,7 +14063,6 @@
           <t>8741157961906</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>10 Pack + (1 FREE)</t>
@@ -14213,7 +14089,6 @@
           <t>TS118_PCK10</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -14262,7 +14137,6 @@
           <t>TS119_WHIT_PCK1</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -14311,7 +14185,6 @@
           <t>TS119_WHIT_PCK10</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -14360,7 +14233,6 @@
           <t>TS119_WHIT_PCK25</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -14409,7 +14281,6 @@
           <t>TS119_WHIT_PCK40</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -14458,7 +14329,6 @@
           <t>TS119_YELW_PCK1</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -14507,7 +14377,6 @@
           <t>TS119_YELW_PCK10</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -14556,7 +14425,6 @@
           <t>TS119_YELW_PCK25</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -14605,7 +14473,6 @@
           <t>TS119_YELW_PCK40</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -14654,7 +14521,6 @@
           <t>TS119_BLUE_PCK1</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -14703,7 +14569,6 @@
           <t>TS119_BLUE_PCK10</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -14752,7 +14617,6 @@
           <t>TS119_BLUE_PCK25</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -14801,7 +14665,6 @@
           <t>TS119_BLUE_PCK40</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -14850,7 +14713,6 @@
           <t>TS119_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -14899,7 +14761,6 @@
           <t>TS119_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -14948,7 +14809,6 @@
           <t>TS119_MLTC_PCK40</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -14997,7 +14857,6 @@
           <t>TS120_CYAN_PCK1</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -15046,7 +14905,6 @@
           <t>TS120_CYAN_PCK10</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -15095,7 +14953,6 @@
           <t>TS120_CYAN_PCK25</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -15144,7 +15001,6 @@
           <t>TS120_BLCK_PCK1</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -15193,7 +15049,6 @@
           <t>TS120_BLCK_PCK10</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -15242,7 +15097,6 @@
           <t>TS120_BLCK_PCK25</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -15291,7 +15145,6 @@
           <t>TS120_ORGN_PCK1</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -15340,7 +15193,6 @@
           <t>TS120_ORGN_PCK10</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -15389,7 +15241,6 @@
           <t>TS120_ORGN_PCK25</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -15438,7 +15289,6 @@
           <t>TS120_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -15487,7 +15337,6 @@
           <t>TS120_MLTC_PCK25</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -15536,7 +15385,6 @@
           <t>TS121_REDD_PCK1</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -15585,7 +15433,6 @@
           <t>TS121_REDD_PCK10</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -15634,7 +15481,6 @@
           <t>TS121_REDD_PCK20</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -15683,7 +15529,6 @@
           <t>TS121_WHIT_PCK1</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -15732,7 +15577,6 @@
           <t>TS121_WHIT_PCK10</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -15781,7 +15625,6 @@
           <t>TS121_WHIT_PCK20</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -15830,7 +15673,6 @@
           <t>TS121_PRPL_PCK1</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -15879,7 +15721,6 @@
           <t>TS121_PRPL_PCK10</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -15928,7 +15769,6 @@
           <t>TS121_PRPL_PCK20</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -15977,7 +15817,6 @@
           <t>TS121_MLTC_PCK10</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -16026,7 +15865,6 @@
           <t>TS121_MLTC_PCK20</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Batch 2: mark all 145 variants linked in CED via bulk CSV
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -8231,7 +8231,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -8273,7 +8273,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -8443,7 +8443,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -8480,7 +8480,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8601,7 +8601,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8638,7 +8638,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -8801,7 +8801,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -8843,7 +8843,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Relisted 2026-10-22, submitted for review (not yet linked in CED)</t>
+          <t>Relisted 2026-10-22, submitted for review and linked in CED (bulk CSV)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -8998,6 +8998,11 @@
           <t>TS104_PINK_PCK1</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9046,6 +9051,11 @@
           <t>TS104_PINK_PCK10</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9094,6 +9104,11 @@
           <t>TS104_PINK_PCK20</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9142,6 +9157,11 @@
           <t>TS104_PINK_PCK30</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9190,6 +9210,11 @@
           <t>TS104_BLUE_PCK1</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9238,6 +9263,11 @@
           <t>TS104_BLUE_PCK10</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9286,6 +9316,11 @@
           <t>TS104_BLUE_PCK20</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9334,6 +9369,11 @@
           <t>TS104_BLUE_PCK30</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9382,6 +9422,11 @@
           <t>TS104_WHIT_PCK1</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9430,6 +9475,11 @@
           <t>TS104_WHIT_PCK10</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9478,6 +9528,11 @@
           <t>TS104_WHIT_PCK20</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9526,6 +9581,11 @@
           <t>TS104_WHIT_PCK30</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9574,6 +9634,11 @@
           <t>TS104_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9622,6 +9687,11 @@
           <t>TS104_MLTC_PCK20</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9670,6 +9740,11 @@
           <t>TS104_MLTC_PCK30</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9718,6 +9793,11 @@
           <t>TS106_YELW_PCK1</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9766,6 +9846,11 @@
           <t>TS106_YELW_PCK10</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9814,6 +9899,11 @@
           <t>TS106_YELW_PCK20</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9862,6 +9952,11 @@
           <t>TS106_YELW_PCK30</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9910,6 +10005,11 @@
           <t>TS106_GREN_PCK1</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9958,6 +10058,11 @@
           <t>TS106_GREN_PCK10</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -10006,6 +10111,11 @@
           <t>TS106_GREN_PCK20</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10054,6 +10164,11 @@
           <t>TS106_GREN_PCK30</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -10102,6 +10217,11 @@
           <t>TS106_PINK_PCK1</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10150,6 +10270,11 @@
           <t>TS106_PINK_PCK10</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10198,6 +10323,11 @@
           <t>TS106_PINK_PCK20</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10246,6 +10376,11 @@
           <t>TS106_PINK_PCK30</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10294,6 +10429,11 @@
           <t>TS106_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10342,6 +10482,11 @@
           <t>TS106_MLTC_PCK20</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10390,6 +10535,11 @@
           <t>TS106_MLTC_PCK30</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10438,6 +10588,11 @@
           <t>TS111_NGRN_PCK1</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10486,6 +10641,11 @@
           <t>TS111_NGRN_PCK10</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10534,6 +10694,11 @@
           <t>TS111_NGRN_PCK25</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10582,6 +10747,11 @@
           <t>TS111_NGRN_PCK40</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10630,6 +10800,11 @@
           <t>TS111_PINK_PCK1</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10678,6 +10853,11 @@
           <t>TS111_PINK_PCK10</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10726,6 +10906,11 @@
           <t>TS111_PINK_PCK25</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10774,6 +10959,11 @@
           <t>TS111_PINK_PCK40</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -10822,6 +11012,11 @@
           <t>TS111_PRPL_PCK1</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -10870,6 +11065,11 @@
           <t>TS111_PRPL_PCK10</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -10918,6 +11118,11 @@
           <t>TS111_PRPL_PCK25</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -10966,6 +11171,11 @@
           <t>TS111_PRPL_PCK40</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -11014,6 +11224,11 @@
           <t>TS111_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -11062,6 +11277,11 @@
           <t>TS111_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -11110,6 +11330,11 @@
           <t>TS111_MLTC_PCK40</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -11158,6 +11383,11 @@
           <t>TS112_REDD_PCK1</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11206,6 +11436,11 @@
           <t>TS112_REDD_PCK10</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11254,6 +11489,11 @@
           <t>TS112_REDD_PCK25</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11302,6 +11542,11 @@
           <t>TS112_WHIT_PCK1</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11350,6 +11595,11 @@
           <t>TS112_WHIT_PCK10</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11398,6 +11648,11 @@
           <t>TS112_WHIT_PCK25</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11446,6 +11701,11 @@
           <t>TS112_GREN_PCK1</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -11494,6 +11754,11 @@
           <t>TS112_GREN_PCK10</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11542,6 +11807,11 @@
           <t>TS112_GREN_PCK25</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11590,6 +11860,11 @@
           <t>TS112_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11638,6 +11913,11 @@
           <t>TS112_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11686,6 +11966,11 @@
           <t>TS113_NGRN_PCK1</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -11734,6 +12019,11 @@
           <t>TS113_NGRN_PCK10</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -11782,6 +12072,11 @@
           <t>TS113_NGRN_PCK25</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11830,6 +12125,11 @@
           <t>TS113_WOVG_PCK1</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -11878,6 +12178,11 @@
           <t>TS113_WOVG_PCK10</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11926,6 +12231,11 @@
           <t>TS113_WOVG_PCK25</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -11974,6 +12284,11 @@
           <t>TS113_BRWN_PCK1</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12022,6 +12337,11 @@
           <t>TS113_BRWN_PCK10</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -12070,6 +12390,11 @@
           <t>TS113_BRWN_PCK25</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -12118,6 +12443,11 @@
           <t>TS113_BLCK_PCK1</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -12166,6 +12496,11 @@
           <t>TS113_BLCK_PCK10</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12214,6 +12549,11 @@
           <t>TS113_BLCK_PCK25</t>
         </is>
       </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12262,6 +12602,11 @@
           <t>TS113_OLVG_PCK1</t>
         </is>
       </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12310,6 +12655,11 @@
           <t>TS113_OLVG_PCK10</t>
         </is>
       </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12358,6 +12708,11 @@
           <t>TS113_OLVG_PCK25</t>
         </is>
       </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12406,6 +12761,11 @@
           <t>TS113_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12454,6 +12814,11 @@
           <t>TS113_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12497,6 +12862,11 @@
           <t>TS114_PCK1</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -12540,6 +12910,11 @@
           <t>TS114_PCK10</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -12583,6 +12958,11 @@
           <t>TS114_PCK25</t>
         </is>
       </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -12631,6 +13011,11 @@
           <t>TS115_YELW_PCK1</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -12679,6 +13064,11 @@
           <t>TS115_YELW_PCK10</t>
         </is>
       </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -12727,6 +13117,11 @@
           <t>TS115_YELW_PCK25</t>
         </is>
       </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -12775,6 +13170,11 @@
           <t>TS115_YELW_PCK40</t>
         </is>
       </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -12823,6 +13223,11 @@
           <t>TS115_ORGN_PCK1</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -12871,6 +13276,11 @@
           <t>TS115_ORGN_PCK10</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -12919,6 +13329,11 @@
           <t>TS115_ORGN_PCK25</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -12967,6 +13382,11 @@
           <t>TS115_ORGN_PCK40</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13015,6 +13435,11 @@
           <t>TS115_WHIT_PCK1</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13063,6 +13488,11 @@
           <t>TS115_WHIT_PCK10</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -13111,6 +13541,11 @@
           <t>TS115_WHIT_PCK25</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13159,6 +13594,11 @@
           <t>TS115_WHIT_PCK40</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -13207,6 +13647,11 @@
           <t>TS115_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -13255,6 +13700,11 @@
           <t>TS115_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -13303,6 +13753,11 @@
           <t>TS115_MLTC_PCK40</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -13351,6 +13806,11 @@
           <t>TS116_SLPL_PCK1</t>
         </is>
       </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13399,6 +13859,11 @@
           <t>TS116_SLPL_PCK10</t>
         </is>
       </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -13447,6 +13912,11 @@
           <t>TS116_SLPL_PCK25</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -13495,6 +13965,11 @@
           <t>TS116_PINK_PCK1</t>
         </is>
       </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -13543,6 +14018,11 @@
           <t>TS116_PINK_PCK10</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13591,6 +14071,11 @@
           <t>TS116_PINK_PCK25</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -13639,6 +14124,11 @@
           <t>TS116_BLCK_PCK1</t>
         </is>
       </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -13687,6 +14177,11 @@
           <t>TS116_BLCK_PCK10</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13735,6 +14230,11 @@
           <t>TS116_BLCK_PCK25</t>
         </is>
       </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -13783,6 +14283,11 @@
           <t>TS116_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -13831,6 +14336,11 @@
           <t>TS116_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -13874,6 +14384,11 @@
           <t>TS117_PCK1</t>
         </is>
       </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -13917,6 +14432,11 @@
           <t>TS117_PCK10</t>
         </is>
       </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -13960,6 +14480,11 @@
           <t>TS117_PCK25</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -14003,6 +14528,11 @@
           <t>TS118_PCK1</t>
         </is>
       </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -14046,6 +14576,11 @@
           <t>TS118_PCK5</t>
         </is>
       </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -14089,6 +14624,11 @@
           <t>TS118_PCK10</t>
         </is>
       </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -14137,6 +14677,11 @@
           <t>TS119_WHIT_PCK1</t>
         </is>
       </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -14185,6 +14730,11 @@
           <t>TS119_WHIT_PCK10</t>
         </is>
       </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -14233,6 +14783,11 @@
           <t>TS119_WHIT_PCK25</t>
         </is>
       </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -14281,6 +14836,11 @@
           <t>TS119_WHIT_PCK40</t>
         </is>
       </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -14329,6 +14889,11 @@
           <t>TS119_YELW_PCK1</t>
         </is>
       </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -14377,6 +14942,11 @@
           <t>TS119_YELW_PCK10</t>
         </is>
       </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -14425,6 +14995,11 @@
           <t>TS119_YELW_PCK25</t>
         </is>
       </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -14473,6 +15048,11 @@
           <t>TS119_YELW_PCK40</t>
         </is>
       </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -14521,6 +15101,11 @@
           <t>TS119_BLUE_PCK1</t>
         </is>
       </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -14569,6 +15154,11 @@
           <t>TS119_BLUE_PCK10</t>
         </is>
       </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -14617,6 +15207,11 @@
           <t>TS119_BLUE_PCK25</t>
         </is>
       </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -14665,6 +15260,11 @@
           <t>TS119_BLUE_PCK40</t>
         </is>
       </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -14713,6 +15313,11 @@
           <t>TS119_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -14761,6 +15366,11 @@
           <t>TS119_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -14809,6 +15419,11 @@
           <t>TS119_MLTC_PCK40</t>
         </is>
       </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -14857,6 +15472,11 @@
           <t>TS120_CYAN_PCK1</t>
         </is>
       </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -14905,6 +15525,11 @@
           <t>TS120_CYAN_PCK10</t>
         </is>
       </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -14953,6 +15578,11 @@
           <t>TS120_CYAN_PCK25</t>
         </is>
       </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -15001,6 +15631,11 @@
           <t>TS120_BLCK_PCK1</t>
         </is>
       </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -15049,6 +15684,11 @@
           <t>TS120_BLCK_PCK10</t>
         </is>
       </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -15097,6 +15737,11 @@
           <t>TS120_BLCK_PCK25</t>
         </is>
       </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -15145,6 +15790,11 @@
           <t>TS120_ORGN_PCK1</t>
         </is>
       </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -15193,6 +15843,11 @@
           <t>TS120_ORGN_PCK10</t>
         </is>
       </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -15241,6 +15896,11 @@
           <t>TS120_ORGN_PCK25</t>
         </is>
       </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -15289,6 +15949,11 @@
           <t>TS120_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -15337,6 +16002,11 @@
           <t>TS120_MLTC_PCK25</t>
         </is>
       </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -15385,6 +16055,11 @@
           <t>TS121_REDD_PCK1</t>
         </is>
       </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -15433,6 +16108,11 @@
           <t>TS121_REDD_PCK10</t>
         </is>
       </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -15481,6 +16161,11 @@
           <t>TS121_REDD_PCK20</t>
         </is>
       </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -15529,6 +16214,11 @@
           <t>TS121_WHIT_PCK1</t>
         </is>
       </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -15577,6 +16267,11 @@
           <t>TS121_WHIT_PCK10</t>
         </is>
       </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -15625,6 +16320,11 @@
           <t>TS121_WHIT_PCK20</t>
         </is>
       </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -15673,6 +16373,11 @@
           <t>TS121_PRPL_PCK1</t>
         </is>
       </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -15721,6 +16426,11 @@
           <t>TS121_PRPL_PCK10</t>
         </is>
       </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -15769,6 +16479,11 @@
           <t>TS121_PRPL_PCK20</t>
         </is>
       </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -15817,6 +16532,11 @@
           <t>TS121_MLTC_PCK10</t>
         </is>
       </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -15863,6 +16583,11 @@
       <c r="J146" t="inlineStr">
         <is>
           <t>TS121_MLTC_PCK20</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Yes (bulk CSV 2026-10-22)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TikTok cleanup batch 3: log new product IDs, all 59 submitted for review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TikTok_Cleanup/TikTok_Pilot_5.xlsx
+++ b/TikTok_Cleanup/TikTok_Pilot_5.xlsx
@@ -27757,7 +27757,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -27768,6 +27768,11 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>&lt;p&gt;Bold bubble lettering for the ravers who are always ready to send it, 3D printed and mounted on a bouncy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Blue, Pink-Blue, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1732780426617459670</t>
         </is>
       </c>
     </row>
@@ -27789,7 +27794,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -27800,6 +27805,11 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>&lt;p&gt;A proud lion crest rave sprout for the emotional, soaring side of bass music, 3D printed in warm festival colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Red, Yellow, Orange, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1732780426617000918</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -27826,7 +27836,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -27837,6 +27847,11 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>&lt;p&gt;A mischievous masked raccoon rave sprout for the late-night crowd, 3D printed and ready to trade.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Black, Purple, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1732780426616083414</t>
         </is>
       </c>
     </row>
@@ -27858,7 +27873,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -27869,6 +27884,11 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>&lt;p&gt;Where soaring melodies meet heavy drops, this two-tone rave sprout is 3D printed for fans of both worlds.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: White-Black, Black, Green-White, Neon Green, Orange, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1732780426616804310</t>
         </is>
       </c>
     </row>
@@ -27890,7 +27910,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -27901,6 +27921,11 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>&lt;p&gt;A funky bear rave sprout full of good-vibes energy, 3D printed and mounted on a strong spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Blue, Yellow, Pink, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1732780426616869846</t>
         </is>
       </c>
     </row>
@@ -27922,7 +27947,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -27933,6 +27958,11 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>&lt;p&gt;Groovy script lettering for the soulful, funky side of the festival, 3D printed in bright colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Blue, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1732780426616148950</t>
         </is>
       </c>
     </row>
@@ -27954,7 +27984,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -27965,6 +27995,11 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>&lt;p&gt;A charged-up lightning bolt rave sprout in shades of green, 3D printed and built for multi-day camping festivals.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Dark Green, Green, Neon Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1732780426616935382</t>
         </is>
       </c>
     </row>
@@ -27986,7 +28021,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -27997,6 +28032,11 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>&lt;p&gt;Clean lettering for the house and tech house crowd, 3D printed and mounted on a bouncy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Aqua, Black, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 10 Pack, 20 Pack, 30 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1732780426614969302</t>
         </is>
       </c>
     </row>
@@ -28018,7 +28058,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -28029,6 +28069,11 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>&lt;p&gt;A woodland coin rave sprout in earthy greens and gold, made for magical nights under the stars.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Green, Olive Green, Gold, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1732780426618246102</t>
         </is>
       </c>
     </row>
@@ -28050,7 +28095,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -28061,6 +28106,11 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>&lt;p&gt;Earthy lettering in green, brown and black for the campground crew, 3D printed and ready to trade.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Green, Brown, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1732780426617066454</t>
         </is>
       </c>
     </row>
@@ -28082,7 +28132,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -28093,6 +28143,11 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>&lt;p&gt;Bold lettering for the headbangers who live for the heaviest drops, 3D printed and built for the pit.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, Green, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 10 Pack, 20 Pack, 30 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1732780426618573782</t>
         </is>
       </c>
     </row>
@@ -28114,7 +28169,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -28125,6 +28180,11 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of woodland-themed rave sprouts, perfect for gifting your whole camp or trading all weekend.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 11 Sprout Bundle, 22 Sprout Bundle, 33 Sprout Bundle, 56 Sprout Bundle, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1732780426616542166</t>
         </is>
       </c>
     </row>
@@ -28146,7 +28206,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -28157,6 +28217,11 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>&lt;p&gt;An archer crest rave sprout with storybook woodland charm, 3D printed and mounted on a strong spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Pink, Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1732780426618639318</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -28183,7 +28248,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -28194,6 +28259,11 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>&lt;p&gt;A little retro TV buddy that rides on your hat all weekend, 3D printed in detail for bass music fans.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Single design, 3D printed in detail&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 3 Pack, 5 Pack, 10 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1732780426616607702</t>
         </is>
       </c>
     </row>
@@ -28215,7 +28285,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -28226,6 +28296,11 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of spooky zombie-themed rave sprouts for Halloween raves and horror-loving bassheads.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 11 Sprout Bundle, 22 Sprout Bundle, 33 Sprout Bundle, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1732780426617656278</t>
         </is>
       </c>
     </row>
@@ -28247,7 +28322,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -28258,6 +28333,11 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>&lt;p&gt;A spooky zombie rave sprout for Halloween raves and haunted dance floors, 3D printed and ready to trade.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Single design, 3D printed in detail&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1732780426616673238</t>
         </is>
       </c>
     </row>
@@ -28279,7 +28359,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -28290,6 +28370,11 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>&lt;p&gt;An out-of-this-world alien head rave sprout for the spaced-out bass crowd, 3D printed in bold colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Turquoise, Purple, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1732780426615034838</t>
         </is>
       </c>
     </row>
@@ -28311,7 +28396,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -28322,6 +28407,11 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>&lt;p&gt;A dreamy cosmic rave sprout for the psychedelic, glitch-hop side of the festival, 3D printed in soft neon tones.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Blue, Purple, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1732780426616280022</t>
         </is>
       </c>
     </row>
@@ -28343,7 +28433,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -28354,6 +28444,11 @@
       <c r="F20" t="inlineStr">
         <is>
           <t>&lt;p&gt;A mind-bending psychedelic rave sprout for trippy bass sets, 3D printed and mounted on a metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Dark Blue, White, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1732780426616214486</t>
         </is>
       </c>
     </row>
@@ -28375,7 +28470,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -28386,6 +28481,11 @@
       <c r="F21" t="inlineStr">
         <is>
           <t>&lt;p&gt;An undead rave sprout for horror fans and Halloween ravers, 3D printed in bright neon colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Yellow, Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1732780426615493590</t>
         </is>
       </c>
     </row>
@@ -28407,7 +28507,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -28418,6 +28518,11 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>&lt;p&gt;A zombie outbreak rave sprout for spooky season raves, 3D printed and ready to spread through your crew.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Orange, Blue, Yellow, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1732780426617721814</t>
         </is>
       </c>
     </row>
@@ -28439,7 +28544,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -28450,6 +28555,11 @@
       <c r="F23" t="inlineStr">
         <is>
           <t>&lt;p&gt;A whimsical top hat tea party rave sprout for storybook-themed festivals, 3D printed in bold colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, Black, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1732780426617131990</t>
         </is>
       </c>
     </row>
@@ -28471,7 +28581,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -28482,6 +28592,11 @@
       <c r="F24" t="inlineStr">
         <is>
           <t>&lt;p&gt;A groovy rave sprout for the tech house dance floor, 3D printed and mounted on a bouncy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Orange, White, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1732780426616345558</t>
         </is>
       </c>
     </row>
@@ -28503,7 +28618,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -28514,6 +28629,11 @@
       <c r="F25" t="inlineStr">
         <is>
           <t>&lt;p&gt;A dark, mysterious rave sprout for the deep bass and techno crowd, 3D printed in punchy neon colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Red, Neon Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>1732780426615559126</t>
         </is>
       </c>
     </row>
@@ -28535,7 +28655,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -28546,6 +28666,11 @@
       <c r="F26" t="inlineStr">
         <is>
           <t>&lt;p&gt;Turned all the way up, this full volume rave sprout is 3D printed for the loudest sets of the weekend.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Green, Red, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>1732780426616411094</t>
         </is>
       </c>
     </row>
@@ -28567,7 +28692,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -28578,6 +28703,11 @@
       <c r="F27" t="inlineStr">
         <is>
           <t>&lt;p&gt;Smooth lettering for the melodic house crowd, 3D printed in cool purples and blues.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, Cyan, Light Blue, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>1732780426618311638</t>
         </is>
       </c>
     </row>
@@ -28599,7 +28729,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -28610,6 +28740,11 @@
       <c r="F28" t="inlineStr">
         <is>
           <t>&lt;p&gt;A max energy rave sprout in fiery colors for high-octane dubstep sets, 3D printed and built to last.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Orange, Red, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>1732780426617197526</t>
         </is>
       </c>
     </row>
@@ -28631,7 +28766,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -28642,6 +28777,11 @@
       <c r="F29" t="inlineStr">
         <is>
           <t>&lt;p&gt;A soaring bird rave sprout for the emotional, singalong moments, 3D printed in sunset colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, Red, Orange, Yellow, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1732780426615821270</t>
         </is>
       </c>
     </row>
@@ -28663,7 +28803,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -28674,6 +28814,11 @@
       <c r="F30" t="inlineStr">
         <is>
           <t>&lt;p&gt;Classic theater masks reimagined as a rave sprout for the dramatic bass crowd, 3D printed in bold colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Neon Green, Black, Orange, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>1732780426617525206</t>
         </is>
       </c>
     </row>
@@ -28695,7 +28840,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -28706,6 +28851,11 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>&lt;p&gt;A skull beats rave sprout for the deep bass faithful, 3D printed and mounted on a strong spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Purple, Neon Green, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>1732780426615886806</t>
         </is>
       </c>
     </row>
@@ -28727,7 +28877,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -28738,6 +28888,11 @@
       <c r="F32" t="inlineStr">
         <is>
           <t>&lt;p&gt;A groovy bass rave sprout for funky, wobbly dance floors, 3D printed in bright colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Pink, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>1732780426615231446</t>
         </is>
       </c>
     </row>
@@ -28759,7 +28914,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -28770,6 +28925,11 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>&lt;p&gt;A 3D spinning bird rave sprout that looks great from every angle, printed in detail for melodic bass fans.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Single design, 3D printed in detail&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 5 Pack, 11 Pack, 22 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>1732780426618442710</t>
         </is>
       </c>
     </row>
@@ -28791,7 +28951,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -28802,6 +28962,11 @@
       <c r="F34" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of melodic bass rave sprouts, perfect for gifting and trading with your whole crew.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 11 Sprout Bundle, 27 Sprout Bundle, 53 Sprout Bundle, 105 Sprout Bundle, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>1732780426615296982</t>
         </is>
       </c>
     </row>
@@ -28823,7 +28988,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -28834,6 +28999,11 @@
       <c r="F35" t="inlineStr">
         <is>
           <t>&lt;p&gt;A detailed 3D bird head rave sprout for melodic bass lovers, printed and mounted on a bouncy spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Single design, 3D printed in detail&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 5 Pack, 11 Pack, 22 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>1732780426615362518</t>
         </is>
       </c>
     </row>
@@ -28855,7 +29025,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -28866,6 +29036,11 @@
       <c r="F36" t="inlineStr">
         <is>
           <t>&lt;p&gt;Rainbow lettering for the bass music faithful, 3D printed and mounted on a bouncy metal spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Rainbow, White, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>1732780426615100374</t>
         </is>
       </c>
     </row>
@@ -28887,7 +29062,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -28898,6 +29073,11 @@
       <c r="F37" t="inlineStr">
         <is>
           <t>&lt;p&gt;A neon bones rave sprout that glows with funky energy, 3D printed in electric colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Turquoise, Cyber Pink, Purple, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1732780426618377174</t>
         </is>
       </c>
     </row>
@@ -28919,7 +29099,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -28930,6 +29110,11 @@
       <c r="F38" t="inlineStr">
         <is>
           <t>&lt;p&gt;A spooky coffin casket rave sprout for dark bass nights, 3D printed and mounted on a strong spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Yellow, Orange, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>1732780426615690198</t>
         </is>
       </c>
     </row>
@@ -28951,7 +29136,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -28962,6 +29147,11 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>&lt;p&gt;Where heavy metal meets heavy bass, this rave sprout is 3D printed for the loudest headbangers.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Gold, Red, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>1732780426618704854</t>
         </is>
       </c>
     </row>
@@ -28983,7 +29173,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -28994,6 +29184,11 @@
       <c r="F40" t="inlineStr">
         <is>
           <t>&lt;p&gt;A dark wings rave sprout for the deep riddim crowd, 3D printed and mounted on a bouncy spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, White, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>1732780426618115030</t>
         </is>
       </c>
     </row>
@@ -29015,7 +29210,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -29026,6 +29221,11 @@
       <c r="F41" t="inlineStr">
         <is>
           <t>&lt;p&gt;A funk and soul rave sprout for groovy, feel-good sets, 3D printed in cool blues and purples.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Light Blue, Purple, Cyan, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>1732780426616738774</t>
         </is>
       </c>
     </row>
@@ -29047,7 +29247,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -29058,6 +29258,11 @@
       <c r="F42" t="inlineStr">
         <is>
           <t>&lt;p&gt;A neon bass rave sprout that pops under the lights, 3D printed and ready to trade all weekend.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Neon Green, Yellow, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>1732780426617787350</t>
         </is>
       </c>
     </row>
@@ -29079,7 +29284,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -29090,6 +29295,11 @@
       <c r="F43" t="inlineStr">
         <is>
           <t>&lt;p&gt;An electro pop rave sprout for big-room singalongs, 3D printed in bright candy colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Cyber Pink, Purple, Yellow, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>1732780426617263062</t>
         </is>
       </c>
     </row>
@@ -29111,7 +29321,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -29122,6 +29332,11 @@
       <c r="F44" t="inlineStr">
         <is>
           <t>&lt;p&gt;A dark riddim rave sprout for the heaviest sets of the night, 3D printed and built for the pit.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Red, Purple, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1732780426618049494</t>
         </is>
       </c>
     </row>
@@ -29143,7 +29358,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -29154,6 +29369,11 @@
       <c r="F45" t="inlineStr">
         <is>
           <t>&lt;p&gt;A dirty south wobble rave sprout full of bounce, 3D printed in bright festival colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Orange, Yellow, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 27 Pack, 44 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>1732780426615952342</t>
         </is>
       </c>
     </row>
@@ -29175,7 +29395,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -29186,6 +29406,11 @@
       <c r="F46" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of dinosaur-themed bass festival rave sprouts, made for gifting and trading with your crew.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 11 Sprout Bundle, 22 Sprout Bundle, 33 Sprout Bundle, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>1732780426617590742</t>
         </is>
       </c>
     </row>
@@ -29207,7 +29432,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -29218,6 +29443,11 @@
       <c r="F47" t="inlineStr">
         <is>
           <t>&lt;p&gt;A heavy wobble rave sprout for the dubstep faithful, 3D printed and mounted on a strong spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, Black, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>1732780426615624662</t>
         </is>
       </c>
     </row>
@@ -29239,7 +29469,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -29250,6 +29480,11 @@
       <c r="F48" t="inlineStr">
         <is>
           <t>&lt;p&gt;A retro radio rave sprout for bass music lovers who keep the station locked, 3D printed in classic colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: White, Blue, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>1732780426616017878</t>
         </is>
       </c>
     </row>
@@ -29271,7 +29506,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -29282,6 +29517,11 @@
       <c r="F49" t="inlineStr">
         <is>
           <t>&lt;p&gt;A swamp monster rave sprout for headbangers with a sense of humor, 3D printed in swampy greens and gold.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Green-White, Gold, Green-Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>1732780426617918422</t>
         </is>
       </c>
     </row>
@@ -29303,7 +29543,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -29314,6 +29554,11 @@
       <c r="F50" t="inlineStr">
         <is>
           <t>&lt;p&gt;A prehistoric bass rave sprout for dinosaur-loving headbangers, 3D printed and ready to stomp.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Red, Purple, Light Blue, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>1732780426615755734</t>
         </is>
       </c>
     </row>
@@ -29335,7 +29580,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -29346,6 +29591,11 @@
       <c r="F51" t="inlineStr">
         <is>
           <t>&lt;p&gt;A double trouble rave sprout for back-to-back bass sets, 3D printed in bold festival colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Purple, Orange, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>1732780426614903766</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -29372,7 +29622,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -29383,6 +29633,11 @@
       <c r="F52" t="inlineStr">
         <is>
           <t>&lt;p&gt;A bass stage rave sprout for the front-row crowd, 3D printed and mounted on a bouncy spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Neon Green, Orange, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>1732780426618180566</t>
         </is>
       </c>
     </row>
@@ -29404,7 +29659,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -29415,6 +29670,11 @@
       <c r="F53" t="inlineStr">
         <is>
           <t>&lt;p&gt;A headliner-worthy bass rave sprout for the biggest sets of the weekend, 3D printed in bold colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Blue, Black, Pink, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>1732780426617328598</t>
         </is>
       </c>
     </row>
@@ -29436,7 +29696,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -29447,6 +29707,11 @@
       <c r="F54" t="inlineStr">
         <is>
           <t>&lt;p&gt;A dino wobble rave sprout for prehistoric-level drops, 3D printed and mounted on a strong spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Purple, White, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>1732780426617983958</t>
         </is>
       </c>
     </row>
@@ -29468,7 +29733,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -29479,6 +29744,11 @@
       <c r="F55" t="inlineStr">
         <is>
           <t>&lt;p&gt;A playful breakfast-themed bass rave sprout for the morning-after crowd, 3D printed in fun colors.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Rainbow, Black, White, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>1732780426615428054</t>
         </is>
       </c>
     </row>
@@ -29500,7 +29770,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -29511,6 +29781,11 @@
       <c r="F56" t="inlineStr">
         <is>
           <t>&lt;p&gt;Elegant cursive lettering meets heavy bass in this two-tone rave sprout, 3D printed and ready to trade.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Black-Blue, Yellow-Turquoise, Black-Yellow, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>1732780426618508246</t>
         </is>
       </c>
     </row>
@@ -29532,7 +29807,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -29543,6 +29818,11 @@
       <c r="F57" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of camp-themed rave sprouts for your whole campsite crew, made for gifting and trading.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 11 Sprout Bundle, 22 Sprout Bundle, 33 Sprout Bundle, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>1732780426615165910</t>
         </is>
       </c>
     </row>
@@ -29564,7 +29844,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -29575,6 +29855,11 @@
       <c r="F58" t="inlineStr">
         <is>
           <t>&lt;p&gt;A drum and bass rave sprout for high-tempo dance floors, 3D printed and mounted on a bouncy spring clip.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Colors: Pink, Green, Black, or Multicolor&lt;/li&gt;&lt;li&gt;Packs: 1 Pack, 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>1732780426617394134</t>
         </is>
       </c>
     </row>
@@ -29596,7 +29881,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -29607,6 +29892,11 @@
       <c r="F59" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of dreamy festival rave sprouts, perfect for gifting and trading all weekend.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 11 Pack, 22 Pack, 33 Pack, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>1732780426616476630</t>
         </is>
       </c>
     </row>
@@ -29628,7 +29918,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Upload file built 2026-10-22 (not uploaded yet)</t>
+          <t>Relisted 2026-10-22, submitted for review</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -29639,6 +29929,11 @@
       <c r="F60" t="inlineStr">
         <is>
           <t>&lt;p&gt;An assorted bundle of rave sprouts for summer lakefront festivals, made for gifting and trading with your crew.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong metal spring clip grips hats, hair, bags, and pashminas through every drop&lt;/li&gt;&lt;li&gt;Built-in bead hole turns it into a kandi bracelet, cuff, or necklace piece for trading&lt;/li&gt;&lt;li&gt;Durable 3D printed PLA charm, made to order, built for crowds, heat, and all-night dancing&lt;/li&gt;&lt;li&gt;Assorted designs and colors in every pack&lt;/li&gt;&lt;li&gt;Packs: 13 Sprout Bundle, 26 Sprout Bundle, 39 Sprout Bundle, perfect for gifting and trading with your crew&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Share it. Trade it. Gift it.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>1732780426617852886</t>
         </is>
       </c>
     </row>

</xml_diff>